<commit_message>
Expand requirements coverage and traceability
</commit_message>
<xml_diff>
--- a/docs/manual-tests/workflow_tracker_manual_api_tests.xlsx
+++ b/docs/manual-tests/workflow_tracker_manual_api_tests.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" r:id="R89a421efacfa4b69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-001 Create Item" sheetId="2" r:id="Ra85b8928b7454a3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-002 Bad Owner" sheetId="3" r:id="R8b890dc471604c04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-003 Blank Title" sheetId="4" r:id="R18b86fe5039049f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-004 Valid Status" sheetId="5" r:id="Re139c2e1ed734613"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-005 Invalid Status" sheetId="6" r:id="Rb1d3186ae0614236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-006 Same Status" sheetId="7" r:id="Rcbcd009aace94f81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" r:id="Rb3021b05601744c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-001 Create Item" sheetId="2" r:id="R5db504ce88724fa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-002 Bad Owner" sheetId="3" r:id="Rb12dd45adbda4c5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-003 Blank Title" sheetId="4" r:id="Ra6672cd181e449f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-004 Valid Status" sheetId="5" r:id="R476385399ef14013"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-005 Invalid Status" sheetId="6" r:id="Re08345cef7ab496f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API-006 Same Status" sheetId="7" r:id="R9d2fc66037de4f60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -68,198 +68,42 @@
   <x:borders count="38">
     <x:border/>
     <x:border/>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -704,7 +548,7 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="F4" s="21" t="str">
-        <x:v>POST create + GET persistence check</x:v>
+        <x:v>POST create + timestamp/history + GET persistence check</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -851,7 +695,7 @@
         <x:v>Purpose</x:v>
       </x:c>
       <x:c r="B4" s="36" t="str">
-        <x:v>Verify that POST /api/items creates an item with the supplied values, NEW status, one initial history entry, and a persisted record retrievable by ID.</x:v>
+        <x:v>Verify that POST /api/items creates an item with the supplied values, NEW status, a creation timestamp, one initial history entry, and a persisted record retrievable by ID.</x:v>
       </x:c>
       <x:c r="C4" s="36"/>
       <x:c r="D4" s="36"/>
@@ -930,7 +774,7 @@
       <x:c r="C11" s="56" t="str">
         <x:v>HTTP 200. Response contains at least one owner with an ID.</x:v>
       </x:c>
-      <x:c r="D11" s="56" t="str"/>
+      <x:c r="D11" s="56"/>
       <x:c r="E11" s="57" t="str">
         <x:v>Setup / not coverage</x:v>
       </x:c>
@@ -945,9 +789,9 @@
       <x:c r="C12" s="56" t="str">
         <x:v>HTTP 201. Response contains the supplied title and description, the selected owner ID, status NEW, and exactly one statusHistory entry.</x:v>
       </x:c>
-      <x:c r="D12" s="56" t="str"/>
+      <x:c r="D12" s="56"/>
       <x:c r="E12" s="57" t="str">
-        <x:v>WF-006 AC-5; WF-006 AC-6; WF-001 AC-7; WF-003 AC-7</x:v>
+        <x:v>WF-006 AC-5; WF-006 AC-6; WF-003 AC-7</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="79.19999694824219" hidden="0" customHeight="1">
@@ -955,14 +799,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B13" s="56" t="str">
-        <x:v>Inspect statusHistory[0].</x:v>
+        <x:v>Inspect the created item's creation timestamp in the response.</x:v>
       </x:c>
       <x:c r="C13" s="56" t="str">
-        <x:v>previousStatus is null/blank and newStatus is NEW.</x:v>
-      </x:c>
-      <x:c r="D13" s="56" t="str"/>
+        <x:v>A creation timestamp is present and nonblank, and its value is consistent with the time the item was created.</x:v>
+      </x:c>
+      <x:c r="D13" s="56"/>
       <x:c r="E13" s="57" t="str">
-        <x:v>WF-003 AC-2; WF-003 AC-7</x:v>
+        <x:v>WF-001 AC-7</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="145.1999969482422" hidden="0" customHeight="1">
@@ -970,14 +814,29 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B14" s="59" t="str">
+        <x:v>Inspect statusHistory[0].</x:v>
+      </x:c>
+      <x:c r="C14" s="59" t="str">
+        <x:v>previousStatus is null/blank and newStatus is NEW.</x:v>
+      </x:c>
+      <x:c r="D14" s="59"/>
+      <x:c r="E14" s="60" t="str">
+        <x:v>WF-003 AC-2; WF-003 AC-7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
         <x:v>Record the returned item ID and GET &lt;base_url&gt;/api/items/&lt;item_id&gt;.</x:v>
       </x:c>
-      <x:c r="C14" s="59" t="str">
-        <x:v>HTTP 200. The persisted item has the same title, status NEW, and one history entry.</x:v>
-      </x:c>
-      <x:c r="D14" s="59" t="str"/>
-      <x:c r="E14" s="60" t="str">
-        <x:v>WF-006 AC-7</x:v>
+      <x:c r="C15" t="str">
+        <x:v>HTTP 200. The persisted item has the same title, status NEW, creation timestamp, and one history entry.</x:v>
+      </x:c>
+      <x:c r="D15"/>
+      <x:c r="E15" t="str">
+        <x:v>WF-006 AC-7; WF-001 AC-7</x:v>
       </x:c>
     </x:row>
     <x:row r="16">

</xml_diff>